<commit_message>
Update prototype HTML and SQL for storage packaging enhancements
- Updated index.html to reflect changes in storage packaging values:
  - Modified stylesheet versioning.
  - Added "存储包装方式" column in relevant tables.
  - Updated table rows to include new packaging values.
  - Adjusted form fields to include storage packaging options.

- Altered tables.sql to include a new column for storage packaging:
  - Added `C_ZCCBZ` for storage packaging type in `material_operation_vehicle_config`.
  - Updated unique key constraint to include the new storage packaging column.

- Updated binary file FS(2).xlsx to reflect changes in packaging data.
</commit_message>
<xml_diff>
--- a/aspnet-core/prototype/领用配送接口FS(2).xlsx
+++ b/aspnet-core/prototype/领用配送接口FS(2).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\module-zero-core-template\aspnet-core\prototype\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7CDA271-C138-473E-84D6-945F7EC2FA34}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B18FB07-DF28-44D9-942E-3A9507D7F3B1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6948" tabRatio="669" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6948" tabRatio="669" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目录" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="364">
   <si>
     <t>A-LM-ABAP-WMZC588</t>
   </si>
@@ -1248,6 +1248,26 @@
   </si>
   <si>
     <t>25,0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>5,0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LGORT</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CHAR</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>LGNUM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>3,0</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1520,7 +1540,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1691,6 +1711,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -5048,8 +5074,8 @@
       <c r="D6" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="35" t="s">
-        <v>78</v>
+      <c r="E6" s="63" t="s">
+        <v>359</v>
       </c>
       <c r="F6" s="35" t="s">
         <v>293</v>
@@ -5233,9 +5259,15 @@
       <c r="B13" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
+      <c r="C13" s="64" t="s">
+        <v>360</v>
+      </c>
+      <c r="D13" s="64" t="s">
+        <v>361</v>
+      </c>
+      <c r="E13" s="35" t="s">
+        <v>56</v>
+      </c>
       <c r="F13" s="35"/>
       <c r="G13" s="35"/>
       <c r="H13" s="35"/>
@@ -5254,9 +5286,15 @@
       <c r="B14" s="35" t="s">
         <v>140</v>
       </c>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
+      <c r="C14" s="64" t="s">
+        <v>362</v>
+      </c>
+      <c r="D14" s="63" t="s">
+        <v>361</v>
+      </c>
+      <c r="E14" s="64" t="s">
+        <v>363</v>
+      </c>
       <c r="F14" s="35"/>
       <c r="G14" s="35"/>
       <c r="H14" s="35"/>
@@ -5774,8 +5812,8 @@
       <c r="D6" s="35" t="s">
         <v>66</v>
       </c>
-      <c r="E6" s="35" t="s">
-        <v>78</v>
+      <c r="E6" s="63" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="7" spans="1:15">

</xml_diff>